<commit_message>
Fill HSK1_parts_of_speech_4(151-200).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_4(151-200).xlsx
+++ b/HSK1_parts_of_speech_4(151-200).xlsx
@@ -601,6 +601,11 @@
           <t>слова, речь</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>речь, слова (谈话, 电话里说的话)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +632,16 @@
           <t>плохой, сломанный</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>испортить, сломать (弄坏了 «испортил», 把电视看坏了) — как результативный комплемент</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>плохой, испорченный, сломанный</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +668,16 @@
           <t>возвращать</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>возвращать (还书, 还钱)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>ещё, тоже, однако (还有, 还要)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -684,6 +709,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>возвращаться; поворачивать (回家, 回头)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>для разовых действий и глав/представлений: 一回 «разок», 两回 «два раза»; 回 для глав книг/спектаклей</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -715,6 +750,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ответ (给我一个回答)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>отвечать, отвечать на (回答问题)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -746,6 +791,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>словосочетание: глагол 回 + направительное дополнение 到</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -777,6 +827,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>словосочетание: глагол 回 + существительное 家 (возвращаться домой)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -808,6 +863,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>глагол с направленным дополнением: 回 + 来 (возвращаться сюда); сам 回来 — глагольная конструкция</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -839,6 +899,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>глагол с направленным дополнением: 回 + 去 (возвращаться туда)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -865,6 +930,16 @@
           <t>мочь</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>собрание, встреча (开会 «проводить собрание»)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>мочь, уметь (会开车); знать, владеть (会英语)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -891,6 +966,11 @@
           <t>поезд</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>поезд (火车)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -917,6 +997,11 @@
           <t>аэропорт</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>аэропорт</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -943,6 +1028,11 @@
           <t>билет на самолёт</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>авиабилет</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -969,6 +1059,11 @@
           <t>яйцо</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>яйцо (куриное)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -995,6 +1090,16 @@
           <t>несколько</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>несколько (几个人 «несколько человек», 几天 «несколько дней»)</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>вопросительное: сколько? (几岁? «сколько лет?», 几天? «сколько дней?» — на вопрос отвечает числом)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1021,6 +1126,11 @@
           <t>помнить, записывать</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>помнить, запоминать; записывать, делать пометки (记笔记, 记住)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1047,6 +1157,16 @@
           <t>помнить</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>помнить, помнить (记得他叫名字)</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>часто анализируется как 记 + частица 得 (возможность/результат), но слово устойчиво</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1073,6 +1193,16 @@
           <t>запоминать</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>запомнить, запоминать накрепко (记住这个名字)</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение 住</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1099,6 +1229,11 @@
           <t>дом; семья</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>дом; семья (回家, 家人)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1125,6 +1260,16 @@
           <t>дома (внутри)</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>дом, семья (внутри дома); 家里 «дома, внутри семьи»</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>словосочетание: 家 + локатив 里; иногда местоименное: 他们家</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1151,6 +1296,11 @@
           <t>член семьи</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>член семьи, домашние</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1177,6 +1327,26 @@
           <t>между</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>промежуток, комната (房间, 车间)</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>для помещений: 一间房 «одна комната», 两间车间</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>между; в составе слов: 民间 «в народе», 车间 «цех» (самостоятельный предлог устар.)</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>В составе слов (房间, 时间) или как счётное; предлог 间 в совр. языке устар.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1203,6 +1373,11 @@
           <t>увидеть, встретить</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>видеть, встречать (看见, 见面); быть видимым (见效 «дать эффект»)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1229,6 +1404,11 @@
           <t>встретить</t>
         </is>
       </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>离合词 (глагол+объект): 见 + 面 «повидаться, встретиться»</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1255,6 +1435,11 @@
           <t>обучать</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>учить, обучать (教书, 教你); преподавать</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1281,6 +1466,11 @@
           <t>звать, называть</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>звать, называться (他叫李明); заставлять (叫我做); кричать, звать (叫门, 大叫)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1307,6 +1497,11 @@
           <t>учебный корпус</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>учебный корпус, учебное здание</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1338,6 +1533,11 @@
           <t>старшая сестра</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>старшая сестра</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1364,6 +1564,16 @@
           <t>представлять, знакомить</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>введение, представление (做一个介绍)</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>представлять, знакомить; вводить, рассказывать (介绍情况)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1390,6 +1600,11 @@
           <t>в этом году</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>этот год (今年很好)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1416,6 +1631,11 @@
           <t>сегодня</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>сегодня</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1442,6 +1662,11 @@
           <t>войти</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>входить, вступать (进来, 进去); вводить (进学校); поступать (进料)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1468,6 +1693,11 @@
           <t>войти (сюда)</t>
         </is>
       </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>глагол с направленным дополнением: 进 + 来 (войти сюда)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1494,6 +1724,11 @@
           <t>войти (туда)</t>
         </is>
       </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>глагол с направленным дополнением: 进 + 去 (войти туда)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1520,6 +1755,11 @@
           <t>девять</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>девять (九月, 十九)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1546,6 +1786,11 @@
           <t>тотчас же, только</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>тотчас же, сразу (他就走); именно (就是 «именно так»); только, лишь (就我们三个人 «нас всего трое»)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1572,6 +1817,16 @@
           <t>полагать, ощущать</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>думать, считать, ощущать (我觉得好)</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>слово образовано от 觉 «чувствовать» + 得; лексикализованное глагольное слово</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1598,6 +1853,11 @@
           <t>открывать</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>открывать (开门, 开灯); водить (车) (开车); запускать, начинать (开会, 开工); устраивать (开晚会); вычитать (开药方)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1624,6 +1884,11 @@
           <t>водить машину</t>
         </is>
       </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>словосочетание/离合词: 开 + 车 «водить машину, ехать»</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1650,6 +1915,11 @@
           <t>проводить собрание</t>
         </is>
       </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>离合词: 开 + 会 «проводить/быть на собрании»</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1676,6 +1946,11 @@
           <t>шутить</t>
         </is>
       </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (离合词): 开 + 玩笑 «шутить»</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1702,6 +1977,11 @@
           <t>смотреть</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>смотреть, читать (看书, 看电影); посещать врача (看病); присматривать (看孩子); думать, считать (我看行)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1728,6 +2008,11 @@
           <t>прийти на осмотр</t>
         </is>
       </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>离合词: 看 + 病 «обращаться к врачу, лечиться (приходить на осмотр)»</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1754,6 +2039,16 @@
           <t>увидеть</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>увидеть, заметить (看到他了)</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>глагол 看 + результативное дополнение 到</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1780,6 +2075,16 @@
           <t>видеть, увидеть</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>видеть, увидеть (看见了)</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>глагол 看 + результативное дополнение 见</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1806,6 +2111,11 @@
           <t>тест</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>тестировать, экзаменовать (考学生); проверять, исследовать (考验); сдавать (考试) (考大学)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1832,6 +2142,16 @@
           <t>экзамен</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>экзамен, тест (一场考试)</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>сдавать экзамен; экзаменовать (参加考试)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1858,6 +2178,11 @@
           <t>испытывать жажду</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>испытывать жажду, хотеть пить (我渴了)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1884,6 +2209,16 @@
           <t>урок</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>урок, занятие (上课, 下课); учебный предмет (一门课)</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>для уроков/занятий и учебных предметов: 一课 «один урок», 两课书 «два урока учебника»</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1906,6 +2241,11 @@
         </is>
       </c>
       <c r="I51" t="inlineStr">
+        <is>
+          <t>учебник</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>учебник</t>
         </is>

</xml_diff>